<commit_message>
Método das calculadoras EC2, filtros, somatório e diagramas de vigas
- Verificação EC2 com as fórmulas das calculadoras (Mosley): K/z, 7.6, 9.6 (β, M'), 10.1, 8.1.1
- Filtros na verificação (assinalados, insuficientes, excesso, tipo, texto)
- Somatório dos materiais por tipo de elemento e conferência com os totais da listagem
- Leitura dos diagramas de esforços de vigas em PDF (M, V, T por pórtico e tramo)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/RevB_Pilares_armaduras.xlsx
+++ b/exemplos/RevB_Pilares_armaduras.xlsx
@@ -74,7 +74,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4Ø20+2Ø16</t>
+          <t>4Ø20+4Ø16</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -83,7 +83,7 @@
         </is>
       </c>
       <c r="F4">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5">
@@ -104,7 +104,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6Ø12</t>
+          <t>4Ø16+2Ø12</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -113,7 +113,7 @@
         </is>
       </c>
       <c r="F5">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6">
@@ -224,7 +224,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4Ø25+4Ø20</t>
+          <t>8Ø25</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -233,7 +233,7 @@
         </is>
       </c>
       <c r="F9">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10">
@@ -254,7 +254,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4Ø20</t>
+          <t>4Ø20+2Ø16</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -263,7 +263,7 @@
         </is>
       </c>
       <c r="F10">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11">
@@ -374,7 +374,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4Ø20+2Ø16</t>
+          <t>8Ø20</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="F14">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -524,7 +524,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4Ø20+2Ø16</t>
+          <t>4Ø20+4Ø16</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="F19">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20">
@@ -554,7 +554,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6Ø12</t>
+          <t>4Ø16+2Ø12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="F20">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21">
@@ -704,7 +704,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4Ø20</t>
+          <t>4Ø20+4Ø16</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="F25">
-        <v>99</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26">
@@ -734,7 +734,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>4Ø16+2Ø12</t>
+          <t>4Ø20</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>4Ø16+2Ø12</t>
+          <t>4Ø20</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -833,7 +833,7 @@
         </is>
       </c>
       <c r="F29">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30">

</xml_diff>